<commit_message>
Wrap-up generators (HAZOP, cost estimate, register) + work-in-progress discipline outputs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013qGZUcwwWBAcAEPeh7Toud
</commit_message>
<xml_diff>
--- a/deliverables/02-equipment/CFU-000-ME-LST-001_Equipment-List.xlsx
+++ b/deliverables/02-equipment/CFU-000-ME-LST-001_Equipment-List.xlsx
@@ -566,7 +566,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>135 / 361</t>
+          <t>134 / 361</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -623,7 +623,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>218</t>
+          <t>220</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>302</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>ID 2.6 m (top) / 6.4 m (main) / 3.0 m (boot) x 36.0 m T/T</t>
+          <t>ID 2.6 m (top) / 6.6 m (main) / 3.0 m (boot) x 36.0 m T/T</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>60.8 MW abs. / 67.6 MW fired; 2-cell cabin, 8 passes, 128 rad. tubes 6" x 18.3 m</t>
+          <t>60.7 MW abs. / 67.4 MW fired; 2-cell cabin, 8 passes, 128 rad. tubes 6" x 18.3 m</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -987,7 +987,7 @@
         <v>3</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>60.81</v>
+        <v>60.68</v>
       </c>
       <c r="M9" s="2" t="inlineStr"/>
     </row>
@@ -1014,7 +1014,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>14.7 MW abs. / 16.8 MW fired; 1-cell cabin, 4 passes, 40 rad. tubes 6" x 18.3 m</t>
+          <t>14.7 MW abs. / 16.7 MW fired; 1-cell cabin, 4 passes, 40 rad. tubes 6" x 18.3 m</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1046,7 +1046,7 @@
         <v>3</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>14.74</v>
+        <v>14.69</v>
       </c>
       <c r="M10" s="2" t="inlineStr"/>
     </row>
@@ -1190,7 +1190,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>357 m2 total; 1S x 1P shells</t>
+          <t>359 m2 total; 1S x 1P shells</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr"/>
@@ -1218,7 +1218,7 @@
         <v>3</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>8.1</v>
+        <v>8.09</v>
       </c>
       <c r="M14" s="2" t="inlineStr"/>
     </row>
@@ -1245,13 +1245,13 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>435 m2 total; 1S x 1P shells</t>
+          <t>438 m2 total; 1S x 1P shells</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr"/>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>H 210-&gt;76 / C 56-&gt;75</t>
+          <t>H 212-&gt;76 / C 56-&gt;75</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1273,7 +1273,7 @@
         <v>3</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>6.49</v>
+        <v>6.55</v>
       </c>
       <c r="M15" s="2" t="inlineStr"/>
     </row>
@@ -1300,13 +1300,13 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>811 m2 total; 2S x 1P shells</t>
+          <t>804 m2 total; 2S x 1P shells</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr"/>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>H 221-&gt;95 / C 75-&gt;108</t>
+          <t>H 224-&gt;95 / C 75-&gt;108</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1316,7 +1316,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>250</t>
+          <t>255</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1328,7 +1328,7 @@
         <v>3</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>11.37</v>
+        <v>11.45</v>
       </c>
       <c r="M16" s="2" t="inlineStr"/>
     </row>
@@ -1355,13 +1355,13 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>379 m2 total; 1S x 1P shells</t>
+          <t>378 m2 total; 1S x 1P shells</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr"/>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>H 205-&gt;128 / C 108-&gt;120</t>
+          <t>H 205-&gt;128 / C 108-&gt;121</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1383,7 +1383,7 @@
         <v>3</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>4.45</v>
+        <v>4.44</v>
       </c>
       <c r="M17" s="2" t="inlineStr"/>
     </row>
@@ -1410,13 +1410,13 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>430 m2 total; 1S x 1P shells</t>
+          <t>431 m2 total; 1S x 1P shells</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>H 255-&gt;175 / C 120-&gt;136</t>
+          <t>H 255-&gt;175 / C 121-&gt;136</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1465,13 +1465,13 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>1041 m2 total; 2S x 1P shells</t>
+          <t>1001 m2 total; 2S x 1P shells</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr"/>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>H 238-&gt;158 / C 136-&gt;169</t>
+          <t>H 240-&gt;160 / C 136-&gt;170</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1493,7 +1493,7 @@
         <v>3</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>12.87</v>
+        <v>12.85</v>
       </c>
       <c r="M19" s="2" t="inlineStr"/>
     </row>
@@ -1520,13 +1520,13 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>318 m2 total; 1S x 1P shells</t>
+          <t>324 m2 total; 1S x 1P shells</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>H 292-&gt;205 / C 169-&gt;184</t>
+          <t>H 294-&gt;205 / C 170-&gt;184</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1536,7 +1536,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>325</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1548,7 +1548,7 @@
         <v>6</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>5.7</v>
+        <v>5.83</v>
       </c>
       <c r="M20" s="2" t="inlineStr"/>
     </row>
@@ -1575,7 +1575,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>2155 m2 total; 2S x 2P shells</t>
+          <t>2196 m2 total; 2S x 2P shells</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr"/>
@@ -1603,7 +1603,7 @@
         <v>6</v>
       </c>
       <c r="L21" s="3" t="n">
-        <v>21.21</v>
+        <v>21.14</v>
       </c>
       <c r="M21" s="2" t="inlineStr"/>
     </row>
@@ -1658,7 +1658,7 @@
         <v>6</v>
       </c>
       <c r="L22" s="3" t="n">
-        <v>3.1</v>
+        <v>3.11</v>
       </c>
       <c r="M22" s="2" t="inlineStr"/>
     </row>
@@ -1685,13 +1685,13 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>876 m2 total; 1S x 2P shells</t>
+          <t>886 m2 total; 1S x 2P shells</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr"/>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>H 313-&gt;261 / C 241-&gt;257</t>
+          <t>H 314-&gt;261 / C 241-&gt;258</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1713,7 +1713,7 @@
         <v>6</v>
       </c>
       <c r="L23" s="3" t="n">
-        <v>7.35</v>
+        <v>7.46</v>
       </c>
       <c r="M23" s="2" t="inlineStr"/>
     </row>
@@ -1740,13 +1740,13 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>1098 m2 total; 1S x 2P shells</t>
+          <t>1094 m2 total; 1S x 2P shells</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr"/>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>H 366-&gt;277 / C 257-&gt;274</t>
+          <t>H 366-&gt;278 / C 258-&gt;274</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1768,7 +1768,7 @@
         <v>6</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>7.61</v>
+        <v>7.58</v>
       </c>
       <c r="M24" s="2" t="inlineStr"/>
     </row>
@@ -1795,13 +1795,13 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>233 m2; 1 shell(s)</t>
+          <t>223 m2; 1 shell(s)</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr"/>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>H 261-&gt;223 / C 186-&gt;186</t>
+          <t>H 261-&gt;224 / C 186-&gt;186</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1823,7 +1823,7 @@
         <v>3</v>
       </c>
       <c r="L25" s="3" t="n">
-        <v>5.04</v>
+        <v>4.91</v>
       </c>
       <c r="M25" s="2" t="inlineStr"/>
     </row>
@@ -1850,13 +1850,13 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>645 m2; 1 shell(s)</t>
+          <t>648 m2; 1 shell(s)</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr"/>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>H 277-&gt;175 / C 148-&gt;148</t>
+          <t>H 278-&gt;175 / C 148-&gt;148</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1878,7 +1878,7 @@
         <v>3</v>
       </c>
       <c r="L26" s="3" t="n">
-        <v>7.58</v>
+        <v>7.62</v>
       </c>
       <c r="M26" s="2" t="inlineStr"/>
     </row>
@@ -1933,7 +1933,7 @@
         <v>3</v>
       </c>
       <c r="L27" s="3" t="n">
-        <v>3.37</v>
+        <v>3.38</v>
       </c>
       <c r="M27" s="2" t="inlineStr"/>
     </row>
@@ -1960,7 +1960,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>741 m2; 2 shell(s)</t>
+          <t>740 m2; 2 shell(s)</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr"/>
@@ -1988,7 +1988,7 @@
         <v>3</v>
       </c>
       <c r="L28" s="3" t="n">
-        <v>5.97</v>
+        <v>5.96</v>
       </c>
       <c r="M28" s="2" t="inlineStr"/>
     </row>
@@ -2043,7 +2043,7 @@
         <v>3</v>
       </c>
       <c r="L29" s="3" t="n">
-        <v>8.49</v>
+        <v>8.51</v>
       </c>
       <c r="M29" s="2" t="inlineStr"/>
     </row>
@@ -2345,13 +2345,13 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>1658 m2 bare; 2 bay(s) 6 m x 12 m, 4 fans</t>
+          <t>1667 m2 bare; 2 bay(s) 6 m x 12 m, 4 fans</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr"/>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>135-&gt;60 (air 35-&gt;55)</t>
+          <t>134-&gt;60 (air 35-&gt;55)</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2371,7 +2371,7 @@
       </c>
       <c r="K35" s="2" t="inlineStr"/>
       <c r="L35" s="3" t="n">
-        <v>33.81</v>
+        <v>33.75</v>
       </c>
       <c r="M35" s="2" t="n">
         <v>90</v>
@@ -2510,7 +2510,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>286 m2 bare; 1 bay(s) 6 m x 12 m, 2 fans</t>
+          <t>287 m2 bare; 1 bay(s) 6 m x 12 m, 2 fans</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr"/>
@@ -2536,7 +2536,7 @@
       </c>
       <c r="K38" s="2" t="inlineStr"/>
       <c r="L38" s="3" t="n">
-        <v>6.03</v>
+        <v>6.06</v>
       </c>
       <c r="M38" s="2" t="n">
         <v>30</v>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="K40" s="2" t="inlineStr"/>
       <c r="L40" s="3" t="n">
-        <v>9.619999999999999</v>
+        <v>9.630000000000001</v>
       </c>
       <c r="M40" s="2" t="n">
         <v>45</v>
@@ -2701,7 +2701,7 @@
       </c>
       <c r="K41" s="2" t="inlineStr"/>
       <c r="L41" s="3" t="n">
-        <v>5.8</v>
+        <v>5.81</v>
       </c>
       <c r="M41" s="2" t="n">
         <v>30</v>
@@ -2730,7 +2730,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>404 m2 bare; 1 bay(s) 6 m x 12 m, 2 fans</t>
+          <t>397 m2 bare; 1 bay(s) 6 m x 12 m, 2 fans</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr"/>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="K42" s="2" t="inlineStr"/>
       <c r="L42" s="3" t="n">
-        <v>3.15</v>
+        <v>3.1</v>
       </c>
       <c r="M42" s="2" t="n">
         <v>15</v>
@@ -2785,7 +2785,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>402 m2 bare; 1 bay(s) 6 m x 12 m, 2 fans</t>
+          <t>403 m2 bare; 1 bay(s) 6 m x 12 m, 2 fans</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr"/>
@@ -3353,7 +3353,7 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>load 3021 kg/h, motive MP steam 7855 kg/h (2 x 50 % parallel)</t>
+          <t>load 3020 kg/h, motive MP steam 7852 kg/h (2 x 50 % parallel)</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr"/>
@@ -3592,7 +3592,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>158 m3/h rated @ 102 m</t>
+          <t>159 m3/h rated @ 102 m</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr"/>
@@ -3788,13 +3788,13 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>388 m3/h rated @ 137 m</t>
+          <t>387 m3/h rated @ 138 m</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr"/>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>238</t>
+          <t>240</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr"/>
@@ -3843,7 +3843,7 @@
       <c r="F63" s="2" t="inlineStr"/>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>313</t>
+          <t>314</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr"/>
@@ -3886,13 +3886,13 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>122 m3/h rated @ 147 m</t>
+          <t>122 m3/h rated @ 148 m</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr"/>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>212</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr"/>
@@ -3941,13 +3941,13 @@
       <c r="F65" s="2" t="inlineStr"/>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>292</t>
+          <t>294</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr"/>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>325</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>84 m3/h rated @ 152 m</t>
+          <t>84 m3/h rated @ 153 m</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr"/>
@@ -4327,19 +4327,19 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>202 m3/h rated @ 138 m</t>
+          <t>198 m3/h rated @ 138 m</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr"/>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>221</t>
+          <t>224</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr"/>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>250</t>
+          <t>255</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
@@ -4376,7 +4376,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>392 m3/h rated @ 144 m</t>
+          <t>391 m3/h rated @ 144 m</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr"/>
@@ -4921,7 +4921,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>805.2</v>
+        <v>805.4</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>263</v>
@@ -4930,7 +4930,7 @@
         <v>20</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>136.0607976966045</v>
+        <v>136.3520743392695</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>776</v>
@@ -4939,7 +4939,7 @@
         <v>0.73</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>615.7</v>
+        <v>615.9</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>710</v>
@@ -4972,7 +4972,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>158.3</v>
+        <v>158.6</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>102</v>
@@ -4990,7 +4990,7 @@
         <v>0.67</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>45.9</v>
+        <v>46</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>55</v>
@@ -5023,7 +5023,7 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>179.6</v>
+        <v>179.9</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>232</v>
@@ -5041,7 +5041,7 @@
         <v>0.67</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>118.4</v>
+        <v>118.6</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>160</v>
@@ -5074,7 +5074,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>14.5</v>
+        <v>14.4</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>51</v>
@@ -5125,7 +5125,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>293</v>
+        <v>292.6</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>130</v>
@@ -5134,7 +5134,7 @@
         <v>8</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>153.263408402976</v>
+        <v>152.8292885846183</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>627</v>
@@ -5143,7 +5143,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>94.2</v>
+        <v>94</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>110</v>
@@ -5176,25 +5176,25 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>387.9</v>
+        <v>387.4</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>8</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>238.4964546011054</v>
+        <v>240.0155698591315</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="H8" s="3" t="n">
         <v>0.7</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>122.9</v>
+        <v>122.8</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>160</v>
@@ -5227,7 +5227,7 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>318.3</v>
+        <v>317.9</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>142</v>
@@ -5236,16 +5236,16 @@
         <v>8</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>312.6428096410828</v>
+        <v>313.9004413771325</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>0.6899999999999999</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>101.9</v>
+        <v>101.8</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>132</v>
@@ -5281,16 +5281,16 @@
         <v>121.5</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E10" s="3" t="n">
         <v>9</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>210.0576955067695</v>
+        <v>211.5077376719267</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>0.66</v>
@@ -5329,7 +5329,7 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>150.6</v>
+        <v>151</v>
       </c>
       <c r="D11" s="3" t="n">
         <v>154</v>
@@ -5338,16 +5338,16 @@
         <v>9</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>291.812731884113</v>
+        <v>293.539066420746</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>0.67</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>56.3</v>
+        <v>56.5</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>75</v>
@@ -5380,25 +5380,25 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>83.59999999999999</v>
+        <v>83.8</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E12" s="3" t="n">
         <v>9</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>334.5796577406791</v>
+        <v>334.7436496087009</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>0.65</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>32.3</v>
+        <v>32.4</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>45</v>
@@ -5431,7 +5431,7 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>398.1</v>
+        <v>397.8</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>172</v>
@@ -5440,7 +5440,7 @@
         <v>12</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>348.5796577406791</v>
+        <v>348.7436496087009</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>710</v>
@@ -5449,7 +5449,7 @@
         <v>0.7</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>189</v>
+        <v>188.9</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>250</v>
@@ -5584,7 +5584,7 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>146.2</v>
+        <v>146.3</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>111</v>
@@ -5635,7 +5635,7 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>142.1</v>
+        <v>142.5</v>
       </c>
       <c r="D17" s="3" t="n">
         <v>98</v>
@@ -5644,7 +5644,7 @@
         <v>6</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>152.3756223899362</v>
+        <v>152.3137756213287</v>
       </c>
       <c r="G17" s="3" t="n">
         <v>624</v>
@@ -5737,7 +5737,7 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>201.7</v>
+        <v>198.3</v>
       </c>
       <c r="D19" s="3" t="n">
         <v>138</v>
@@ -5746,16 +5746,16 @@
         <v>10</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>220.5624132856465</v>
+        <v>223.7069906480531</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="H19" s="3" t="n">
         <v>0.68</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>82.59999999999999</v>
+        <v>81.3</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>110</v>
@@ -5788,7 +5788,7 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>392.2</v>
+        <v>391</v>
       </c>
       <c r="D20" s="3" t="n">
         <v>144</v>
@@ -5797,16 +5797,16 @@
         <v>10</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>315.1768033292034</v>
+        <v>314.9938703914651</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="H20" s="3" t="n">
         <v>0.7</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>155.3</v>
+        <v>154.8</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>200</v>
@@ -5848,7 +5848,7 @@
         <v>8</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>378.3139675704387</v>
+        <v>378.4357134139163</v>
       </c>
       <c r="G21" s="3" t="n">
         <v>714</v>
@@ -5890,7 +5890,7 @@
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>195.5</v>
+        <v>195.6</v>
       </c>
       <c r="D22" s="3" t="n">
         <v>187</v>
@@ -5899,7 +5899,7 @@
         <v>14</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>366.3139675704387</v>
+        <v>366.4357134139163</v>
       </c>
       <c r="G22" s="3" t="n">
         <v>761</v>
@@ -6126,19 +6126,19 @@
         </is>
       </c>
       <c r="D2" s="4" t="n">
-        <v>215865</v>
+        <v>216219</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>2.4</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>98</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>51052</v>
+        <v>51101</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -6294,7 +6294,7 @@
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>101893</v>
+        <v>102070</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>13</v>
@@ -6306,7 +6306,7 @@
         <v>54.2</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>7163</v>
+        <v>7175</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
@@ -6378,7 +6378,7 @@
         </is>
       </c>
       <c r="D8" s="4" t="n">
-        <v>76886</v>
+        <v>76867</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>3.5</v>
@@ -6390,7 +6390,7 @@
         <v>81</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>14023</v>
+        <v>14019</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -6546,7 +6546,7 @@
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>32790</v>
+        <v>32789</v>
       </c>
       <c r="E12" s="3" t="n">
         <v>3.5</v>
@@ -6558,7 +6558,7 @@
         <v>60</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>9338</v>
+        <v>9337</v>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
@@ -6720,10 +6720,10 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>8.1</v>
+        <v>8.09</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>1</v>
@@ -6772,10 +6772,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>6.49</v>
+        <v>6.55</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>1</v>
@@ -6784,11 +6784,11 @@
         <v>300</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>0.83</v>
+        <v>0.82</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>H 210-&gt;76 / C 56-&gt;75</t>
+          <t>H 212-&gt;76 / C 56-&gt;75</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -6824,10 +6824,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>11.37</v>
+        <v>11.45</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>811</v>
+        <v>804</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>2</v>
@@ -6840,7 +6840,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>H 221-&gt;95 / C 75-&gt;108</t>
+          <t>H 224-&gt;95 / C 75-&gt;108</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -6876,10 +6876,10 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4.45</v>
+        <v>4.44</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>1</v>
@@ -6892,7 +6892,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>H 205-&gt;128 / C 108-&gt;120</t>
+          <t>H 205-&gt;128 / C 108-&gt;121</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -6931,7 +6931,7 @@
         <v>5.84</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>1</v>
@@ -6944,7 +6944,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>H 255-&gt;175 / C 120-&gt;136</t>
+          <t>H 255-&gt;175 / C 121-&gt;136</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -6980,10 +6980,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>12.87</v>
+        <v>12.85</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>1041</v>
+        <v>1001</v>
       </c>
       <c r="F7" s="2" t="n">
         <v>2</v>
@@ -6992,11 +6992,11 @@
         <v>320</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0.93</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>H 238-&gt;158 / C 136-&gt;169</t>
+          <t>H 240-&gt;160 / C 136-&gt;170</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -7032,10 +7032,10 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>5.7</v>
+        <v>5.83</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>318</v>
+        <v>324</v>
       </c>
       <c r="F8" s="2" t="n">
         <v>1</v>
@@ -7044,11 +7044,11 @@
         <v>290</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.95</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>H 292-&gt;205 / C 169-&gt;184</t>
+          <t>H 294-&gt;205 / C 170-&gt;184</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -7084,10 +7084,10 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>21.21</v>
+        <v>21.14</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>2155</v>
+        <v>2196</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>4</v>
@@ -7136,7 +7136,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>3.1</v>
+        <v>3.11</v>
       </c>
       <c r="E10" s="3" t="n">
         <v>263</v>
@@ -7188,10 +7188,10 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>7.35</v>
+        <v>7.46</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>876</v>
+        <v>886</v>
       </c>
       <c r="F11" s="2" t="n">
         <v>2</v>
@@ -7204,7 +7204,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>H 313-&gt;261 / C 241-&gt;257</t>
+          <t>H 314-&gt;261 / C 241-&gt;258</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -7240,10 +7240,10 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>7.61</v>
+        <v>7.58</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>1098</v>
+        <v>1094</v>
       </c>
       <c r="F12" s="2" t="n">
         <v>2</v>
@@ -7256,7 +7256,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>H 366-&gt;277 / C 257-&gt;274</t>
+          <t>H 366-&gt;278 / C 258-&gt;274</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -7292,10 +7292,10 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>5.04</v>
+        <v>4.91</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="F13" s="2" t="n">
         <v>1</v>
@@ -7306,7 +7306,7 @@
       <c r="H13" s="2" t="inlineStr"/>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>H 261-&gt;223 / C 186-&gt;186</t>
+          <t>H 261-&gt;224 / C 186-&gt;186</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -7342,10 +7342,10 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>7.58</v>
+        <v>7.62</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="F14" s="2" t="n">
         <v>1</v>
@@ -7356,7 +7356,7 @@
       <c r="H14" s="2" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>H 277-&gt;175 / C 148-&gt;148</t>
+          <t>H 278-&gt;175 / C 148-&gt;148</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -7392,7 +7392,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>3.37</v>
+        <v>3.38</v>
       </c>
       <c r="E15" s="3" t="n">
         <v>117</v>
@@ -7442,10 +7442,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>5.97</v>
+        <v>5.96</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="F16" s="2" t="n">
         <v>2</v>
@@ -7492,7 +7492,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>8.49</v>
+        <v>8.51</v>
       </c>
       <c r="E17" s="3" t="n">
         <v>190</v>
@@ -7853,10 +7853,10 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>33.81</v>
+        <v>33.75</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>1658</v>
+        <v>1667</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>2</v>
@@ -7869,7 +7869,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>135-&gt;60 (air 35-&gt;55)</t>
+          <t>134-&gt;60 (air 35-&gt;55)</t>
         </is>
       </c>
     </row>
@@ -7949,10 +7949,10 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>6.03</v>
+        <v>6.06</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>1</v>
@@ -8013,7 +8013,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>9.619999999999999</v>
+        <v>9.630000000000001</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>881</v>
@@ -8045,7 +8045,7 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>5.8</v>
+        <v>5.81</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>401</v>
@@ -8077,10 +8077,10 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>3.15</v>
+        <v>3.1</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>404</v>
+        <v>397</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>1</v>
@@ -8112,7 +8112,7 @@
         <v>6.64</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>1</v>

</xml_diff>